<commit_message>
adjustd tests for now
</commit_message>
<xml_diff>
--- a/documents/backgroundstars_teststars.xlsx
+++ b/documents/backgroundstars_teststars.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andreatanzer/Documents/Space Science/MasterThesis/WALTzER-simulator/documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{106EBF43-3427-3648-A899-74BA91DE4A89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37D1696C-057E-D84D-8D9D-A2D7EB56B343}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19940" yWindow="4800" windowWidth="28040" windowHeight="17180" activeTab="3" xr2:uid="{602D7A17-CB1A-0B47-BD4B-C0D1174FACF0}"/>
+    <workbookView xWindow="16400" yWindow="1700" windowWidth="28040" windowHeight="17180" activeTab="3" xr2:uid="{602D7A17-CB1A-0B47-BD4B-C0D1174FACF0}"/>
   </bookViews>
   <sheets>
     <sheet name="HD_189733" sheetId="2" r:id="rId1"/>

</xml_diff>